<commit_message>
Auto Update 4D backfill 2026-06-21 -> 2026-09-16 — 6 update(s)
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -9080,6 +9080,9 @@
       <c r="AD62" t="n">
         <v>16778</v>
       </c>
+      <c r="AE62" t="n">
+        <v>31340</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -9278,6 +9281,9 @@
       <c r="AD64" t="n">
         <v>10768</v>
       </c>
+      <c r="AE64" t="n">
+        <v>19256</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10573,6 +10579,9 @@
       <c r="AD77" t="n">
         <v>46258</v>
       </c>
+      <c r="AE77" t="n">
+        <v>48705</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -18912,6 +18921,9 @@
       <c r="AD171" t="n">
         <v>4774</v>
       </c>
+      <c r="AE171" t="n">
+        <v>19256</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -18983,6 +18995,9 @@
       <c r="AD172" t="n">
         <v>8486</v>
       </c>
+      <c r="AE172" t="n">
+        <v>19256</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -19212,6 +19227,9 @@
       </c>
       <c r="AD175" t="n">
         <v>6962</v>
+      </c>
+      <c r="AE175" t="n">
+        <v>48705</v>
       </c>
     </row>
     <row r="176">

</xml_diff>

<commit_message>
Auto Update 4D backfill 2026-06-21 -> 2026-09-16 — 2 update(s)
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -5940,6 +5940,9 @@
       <c r="AD25" t="n">
         <v>31203</v>
       </c>
+      <c r="AE25" t="n">
+        <v>33686</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9988,6 +9991,9 @@
       </c>
       <c r="AD70" t="n">
         <v>43654</v>
+      </c>
+      <c r="AE70" t="n">
+        <v>45299</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
Auto Update 4D 2026-09-16 — 5 update(s)
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -14483,6 +14483,9 @@
       <c r="AD118" t="n">
         <v>33050</v>
       </c>
+      <c r="AE118" t="n">
+        <v>34003</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -14585,6 +14588,9 @@
       <c r="AD119" t="n">
         <v>4699</v>
       </c>
+      <c r="AE119" t="n">
+        <v>5279</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -14656,6 +14662,9 @@
       <c r="AD120" t="n">
         <v>30049</v>
       </c>
+      <c r="AE120" t="n">
+        <v>27883</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -14976,6 +14985,9 @@
       <c r="AC124" t="n">
         <v>19748</v>
       </c>
+      <c r="AE124" t="n">
+        <v>5026</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -15313,6 +15325,9 @@
       </c>
       <c r="AD128" t="n">
         <v>20007</v>
+      </c>
+      <c r="AE128" t="n">
+        <v>19814</v>
       </c>
     </row>
     <row r="129">

</xml_diff>

<commit_message>
Copenhagen Half Marathon SEMI 2026 : 43779 finishers
Source utilisateur. Onglets 10K/21K/42K resynchronises depuis ALL,
dashboard regenere (present dans RAW).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -14907,6 +14907,9 @@
       <c r="AC42" t="n">
         <v>31440</v>
       </c>
+      <c r="AD42" t="n">
+        <v>43779</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -43664,6 +43667,9 @@
       <c r="AD78" t="n">
         <v>31440</v>
       </c>
+      <c r="AE78" t="n">
+        <v>43779</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">

</xml_diff>

<commit_message>
Copenhagen Half Marathon SEMI 2026 : correction 43779 -> 39473
Valeur corrigee par l'utilisateur. Ecrasement volontaire de la cellule
deja remplie (la protection SKIP d'update_finishers.py ne couvre pas la
correction d'une valeur existante). La notification du 43779 est corrigee
sur place dans update_log.json plutot que dupliquee.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -14908,7 +14908,7 @@
         <v>31440</v>
       </c>
       <c r="AD42" t="n">
-        <v>43779</v>
+        <v>39473</v>
       </c>
     </row>
     <row r="43">
@@ -43668,7 +43668,7 @@
         <v>31440</v>
       </c>
       <c r="AE78" t="n">
-        <v>43779</v>
+        <v>39473</v>
       </c>
     </row>
     <row r="79">

</xml_diff>

<commit_message>
BMW Berlin Marathon MARATHON 2026 : 50084 finishers + repli 4D elargi
Source utilisateur pour les finishers.

Le mode repli ne retenait que les epreuves dont la cellule finishers etait
vide : des qu'une valeur etait saisie a la main, l'epreuve en sortait et ses
chronos vainqueurs et son temps moyen ne pouvaient plus jamais etre collectes.
Une epreuve reste desormais eligible tant qu'il manque l'une des quatre
donnees (_chronos_deja_remplis, _avg_deja_remplis). 56 epreuves eligibles au
6 octobre contre 15 avant, reparties sur 9 plateformes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -27311,6 +27311,9 @@
       <c r="AC22" t="n">
         <v>48361</v>
       </c>
+      <c r="AD22" t="n">
+        <v>50084</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -27576,6 +27579,9 @@
       </c>
       <c r="AC25" t="n">
         <v>28990</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>30085</v>
       </c>
     </row>
     <row r="26">
@@ -43467,6 +43473,9 @@
       <c r="AD76" t="n">
         <v>48361</v>
       </c>
+      <c r="AE76" t="n">
+        <v>50084</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">

</xml_diff>

<commit_message>
Stockholm Marathon MARATHON 2026 : 18926 finishers
Compte exact par dichotomie sur le classement mikatiming (2025 : 18839).
C'est la cellule ou l'automatisation avait ecrit 25 en septembre, faute de
savoir compter une page pleine sans liens de pagination.

Au passage, chronos_mikatiming() refaisait sa propre construction d'URL et
rejetait les sous-domaines sans point ('stockholm', 'hamburg', 'vienna',
'brighton') : il passe par url_liste_mikatiming comme le reste.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -30763,6 +30763,9 @@
       <c r="AC64" t="n">
         <v>18839</v>
       </c>
+      <c r="AD64" t="n">
+        <v>18926</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -50930,6 +50933,9 @@
       <c r="AD160" t="n">
         <v>18839</v>
       </c>
+      <c r="AE160" t="n">
+        <v>18926</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">

</xml_diff>

<commit_message>
Mikatiming 2026 : temps moyens Vienne, Brighton, Hambourg + finishers alignes sur le classement
Temps moyens calcules sur l'integralite des classements, aucun chrono hors
bornes de plausibilite :
  Vienna City Marathon       04:28:21 (8667 chronos, mediane 04:25:59)
  Brighton Marathon Week end 04:35:12 (14057, mediane 04:29:27)
  Haspa Marathon Hamburg     04:26:21 (15521, mediane 04:22:51)

Finishers 2026 alignes sur le compte exact du classement, comme pour Berlin :
Vienne 8645 -> 8667, Brighton 14049 -> 14057, Hambourg 15550 -> 15521.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -26761,7 +26761,7 @@
         <v>9286</v>
       </c>
       <c r="AD16" t="n">
-        <v>8645</v>
+        <v>8667</v>
       </c>
     </row>
     <row r="17">
@@ -30574,7 +30574,7 @@
         <v>11671</v>
       </c>
       <c r="AD62" t="n">
-        <v>15550</v>
+        <v>15521</v>
       </c>
     </row>
     <row r="63">
@@ -32429,7 +32429,7 @@
         </is>
       </c>
       <c r="AD105" t="n">
-        <v>14049</v>
+        <v>14057</v>
       </c>
     </row>
     <row r="106">
@@ -41187,7 +41187,7 @@
         <v>9286</v>
       </c>
       <c r="AE53" t="n">
-        <v>8645</v>
+        <v>8667</v>
       </c>
     </row>
     <row r="54">
@@ -50734,7 +50734,7 @@
         <v>11671</v>
       </c>
       <c r="AE158" t="n">
-        <v>15550</v>
+        <v>15521</v>
       </c>
     </row>
     <row r="159">
@@ -58069,7 +58069,7 @@
         </is>
       </c>
       <c r="AE358" t="n">
-        <v>14049</v>
+        <v>14057</v>
       </c>
     </row>
     <row r="359">

</xml_diff>

<commit_message>
TCS London Marathon 2026 : temps moyen 04:36:28, finishers 59862
Calcule sur 59857 chronos du classement (5 ecartes par les bornes de
plausibilite, fauteuils). Mediane 04:28:44, 9.157 km/h. Telechargement des
599 pages en 3 minutes grace a la lecture parallele.

Finishers alignes sur le compte exact du classement : 59830 -> 59862.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -26198,7 +26198,7 @@
         <v>56640</v>
       </c>
       <c r="AD10" t="n">
-        <v>59830</v>
+        <v>59862</v>
       </c>
     </row>
     <row r="11">
@@ -39859,7 +39859,7 @@
         <v>56640</v>
       </c>
       <c r="AE38" t="n">
-        <v>59830</v>
+        <v>59862</v>
       </c>
     </row>
     <row r="39">

</xml_diff>

<commit_message>
Pittsburgh : historique marathon seul, Paris 2026 a 57516, repli Athlinks par course
Dick's Pittsburgh Marathon est un evenement multi-distance et l'historique
melangeait le total de l'evenement avec la seule distance marathon. Corrige
depuis le compte par course d'Athlinks :
  2022  16750 -> 2620
  2023  23636 -> 3005
  2024  19748 -> 3593
  2025   vide -> 3786
2026 valait deja 5026, marathon seul, ce qui avait mis l'ecart en evidence.

Marathon de Paris 2026 : 57464 -> 57516, valeur de l'API TimeTo.

Ces chiffres n'etaient pas accessibles au fetcher : la description d'une
edition ne porte les comptes que pour les annees recentes, et le tableau
`races` n'a pas de compteur. L'API alaska.athlinks.com/Events/Race/Api en a
un pour toutes les editions ; elle est ajoutee en repli, avec le meme ciblage
par distance et le meme refus en cas d'ambiguite.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -26298,7 +26298,7 @@
         <v>55499</v>
       </c>
       <c r="AD11" t="n">
-        <v>57464</v>
+        <v>57516</v>
       </c>
     </row>
     <row r="12">
@@ -28715,13 +28715,16 @@
         </is>
       </c>
       <c r="Z38" t="n">
-        <v>16750</v>
+        <v>2620</v>
       </c>
       <c r="AA38" t="n">
-        <v>23636</v>
+        <v>3005</v>
       </c>
       <c r="AB38" t="n">
-        <v>19748</v>
+        <v>3593</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>3786</v>
       </c>
       <c r="AD38" t="n">
         <v>5026</v>
@@ -39964,7 +39967,7 @@
         <v>55499</v>
       </c>
       <c r="AE39" t="n">
-        <v>57464</v>
+        <v>57516</v>
       </c>
     </row>
     <row r="40">
@@ -47961,13 +47964,16 @@
         </is>
       </c>
       <c r="AA124" t="n">
-        <v>16750</v>
+        <v>2620</v>
       </c>
       <c r="AB124" t="n">
-        <v>23636</v>
+        <v>3005</v>
       </c>
       <c r="AC124" t="n">
-        <v>19748</v>
+        <v>3593</v>
+      </c>
+      <c r="AD124" t="n">
+        <v>3786</v>
       </c>
       <c r="AE124" t="n">
         <v>5026</v>

</xml_diff>

<commit_message>
Pittsburgh : vider 2016, 2018 et 2019
14132, 21135 et 20140 ont le meme profil que les valeurs corrigees juste
avant : des totaux d'evenement, toutes distances confondues, la ou le
dashboard tient une ligne par couple (epreuve, distance). Athlinks n'expose
pas ces editions, donc le chiffre du marathon seul n'est pas recuperable.
Une cellule vide vaut mieux qu'un chiffre faux.

L'historique ne porte plus que des comptes marathon : 2620, 3005, 3593,
3786, 5026.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -28695,15 +28695,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="T38" t="n">
-        <v>14132</v>
-      </c>
-      <c r="V38" t="n">
-        <v>21135</v>
-      </c>
-      <c r="W38" t="n">
-        <v>20140</v>
-      </c>
       <c r="X38" t="inlineStr">
         <is>
           <t>-</t>
@@ -47944,15 +47935,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="U124" t="n">
-        <v>14132</v>
-      </c>
-      <c r="W124" t="n">
-        <v>21135</v>
-      </c>
-      <c r="X124" t="n">
-        <v>20140</v>
-      </c>
       <c r="Y124" t="inlineStr">
         <is>
           <t>-</t>

</xml_diff>

<commit_message>
Marine Corps Marathon 2025 : 28990 -> 30085
Compte Athlinks de la course « Marathon », confirme par l'utilisateur. Le
bond par rapport a 2024 (16168) tient a la 50e edition, pas a un total
d'evenement comme je le soupconnais.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -27578,7 +27578,7 @@
         <v>16168</v>
       </c>
       <c r="AC25" t="n">
-        <v>28990</v>
+        <v>30085</v>
       </c>
     </row>
     <row r="26">
@@ -44364,7 +44364,7 @@
         <v>16168</v>
       </c>
       <c r="AD85" t="n">
-        <v>28990</v>
+        <v>30085</v>
       </c>
     </row>
     <row r="86">

</xml_diff>

<commit_message>
Auto Update 4D 2026-10-06 — 6 update(s)
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -45135,6 +45135,9 @@
       <c r="AD92" t="n">
         <v>16280</v>
       </c>
+      <c r="AE92" t="n">
+        <v>15862</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -45771,6 +45774,9 @@
       <c r="AD99" t="n">
         <v>11338</v>
       </c>
+      <c r="AE99" t="n">
+        <v>10051</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -50836,6 +50842,9 @@
       <c r="AD159" t="n">
         <v>12319</v>
       </c>
+      <c r="AE159" t="n">
+        <v>12327</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -53796,6 +53805,9 @@
       </c>
       <c r="AD190" t="n">
         <v>5145</v>
+      </c>
+      <c r="AE190" t="n">
+        <v>5591</v>
       </c>
     </row>
     <row r="191">

</xml_diff>

<commit_message>
Vancouver Sun Run 10KM 2026 : 45408 finishers
Source utilisateur. La reprise post-covid se poursuit : 25108 en 2023, puis
34990, 39385 et 45408. L'epreuve retrouve son niveau d'avant 2020 (41645 en
2018) sans encore atteindre son record de 48904 en 2012.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -1164,6 +1164,9 @@
       <c r="AC7" t="n">
         <v>39385</v>
       </c>
+      <c r="AD7" t="n">
+        <v>45408</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -40109,6 +40112,9 @@
       <c r="AD40" t="n">
         <v>39385</v>
       </c>
+      <c r="AE40" t="n">
+        <v>45408</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">

</xml_diff>

<commit_message>
SKECHERS Hot Chocolate Run - Philadelphia : renommage et partenaire titre
- "Hot Chocolate Run" -> "SKECHERS Hot Chocolate Run - Philadelphia"
  (Excel ALL + onglets distance, event_countries.json, event_organizers.json)
- Partenaire titre : Skechers, 2026
- Marque ecrite "Skechers", la casse deja en base, pour ne pas creer de
  doublon avec son partenariat official sur Bay to Breakers

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDRDdaoD47bJRT7WbM1up5
</commit_message>
<xml_diff>
--- a/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
+++ b/Suivi_Finishers_Monde_10k_-_21k_-_42k_HISTORIQUE.xlsx
@@ -3838,7 +3838,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Hot Chocolate Run</t>
+          <t>SKECHERS Hot Chocolate Run - Philadelphia</t>
         </is>
       </c>
     </row>
@@ -54878,7 +54878,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Hot Chocolate Run</t>
+          <t>SKECHERS Hot Chocolate Run - Philadelphia</t>
         </is>
       </c>
     </row>
@@ -54900,7 +54900,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Hot Chocolate Run</t>
+          <t>SKECHERS Hot Chocolate Run - Philadelphia</t>
         </is>
       </c>
     </row>
@@ -54922,7 +54922,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Hot Chocolate Run</t>
+          <t>SKECHERS Hot Chocolate Run - Philadelphia</t>
         </is>
       </c>
       <c r="AD224" t="n">

</xml_diff>